<commit_message>
Fix L400 latest production date DAX
Co-authored-by: Copilot <223556219+Copilot@users.noreply.github.com>

Copilot-Session: cd1b0cf6-8323-47ad-9dc4-9bbf1f85cabf
</commit_message>
<xml_diff>
--- a/eval/eval_set_L400.xlsx
+++ b/eval/eval_set_L400.xlsx
@@ -708,7 +708,7 @@
       <c r="E3" s="3" t="inlineStr">
         <is>
           <t>DEFINE
-    VAR _LatestDate = [Latest Date]
+    VAR _LatestDate = CALCULATE(MAX(ProductionLog[Date]), REMOVEFILTERS())
     VAR _Last30Days =
         FILTER(
             ALL('Date'[Date]),
@@ -758,7 +758,7 @@
       <c r="E4" s="3" t="inlineStr">
         <is>
           <t>DEFINE
-    VAR _LatestDate = [Latest Date]
+    VAR _LatestDate = CALCULATE(MAX(ProductionLog[Date]), REMOVEFILTERS())
     VAR _CurrentYear = YEAR(_LatestDate)
     VAR _StartOfYear = DATE(_CurrentYear, 1, 1)
     VAR _StartOfYearPY = DATE(_CurrentYear - 1, 1, 1)
@@ -827,7 +827,7 @@
       <c r="E5" s="3" t="inlineStr">
         <is>
           <t>DEFINE
-    VAR _LatestDate = [Latest Date]
+    VAR _LatestDate = CALCULATE(MAX(ProductionLog[Date]), REMOVEFILTERS())
     VAR _Last6WeeksDates =
         DATESINPERIOD('Date'[Date], _LatestDate, -42, DAY)
 EVALUATE
@@ -918,7 +918,7 @@
           <t>DEFINE
     VAR _TPFilter =
         TREATAS({"Pumps", "Turbines"}, 'Products'[Category])
-    VAR _LatestDate = [Latest Date]
+    VAR _LatestDate = CALCULATE(MAX(ProductionLog[Date]), REMOVEFILTERS())
     VAR _ThisYear = YEAR(_LatestDate)
     VAR _PrevYear = _ThisYear - 1
     VAR _OEE_ThisYear =
@@ -973,7 +973,7 @@
       <c r="E8" s="3" t="inlineStr">
         <is>
           <t>DEFINE
-    VAR _LatestDate = [Latest Date]
+    VAR _LatestDate = CALCULATE(MAX(ProductionLog[Date]), REMOVEFILTERS())
     VAR _StartDate = _LatestDate - 29
     VAR _Last30Days =
         FILTER(
@@ -1035,7 +1035,7 @@
       <c r="E9" s="3" t="inlineStr">
         <is>
           <t>DEFINE
-    VAR _LatestDate = [Latest Date]
+    VAR _LatestDate = CALCULATE(MAX(ProductionLog[Date]), REMOVEFILTERS())
     VAR _Last30Days =
         FILTER(
             ALL('Date'[Date]),
@@ -1085,7 +1085,7 @@
       <c r="E10" s="3" t="inlineStr">
         <is>
           <t>DEFINE
-    VAR _LatestDate = [Latest Date]
+    VAR _LatestDate = CALCULATE(MAX(ProductionLog[Date]), REMOVEFILTERS())
     VAR _Last30Days =
         FILTER(
             ALL('Date'[Date]),

</xml_diff>

<commit_message>
Update L400 evaluation test questions
Co-authored-by: Copilot <223556219+Copilot@users.noreply.github.com>

Copilot-Session: cd1b0cf6-8323-47ad-9dc4-9bbf1f85cabf
</commit_message>
<xml_diff>
--- a/eval/eval_set_L400.xlsx
+++ b/eval/eval_set_L400.xlsx
@@ -2,9 +2,8 @@
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <workbookPr/>
-  <workbookProtection/>
   <bookViews>
-    <workbookView visibility="visible" minimized="0" showHorizontalScroll="1" showVerticalScroll="1" showSheetTabs="1" tabRatio="600" firstSheet="0" activeTab="0" autoFilterDateGrouping="1"/>
+    <workbookView visibility="visible" minimized="0" showHorizontalScroll="1" showVerticalScroll="1" showSheetTabs="1" xWindow="-114" yWindow="-114" windowWidth="49274" windowHeight="20060" tabRatio="600" firstSheet="0" activeTab="1" autoFilterDateGrouping="1"/>
   </bookViews>
   <sheets>
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="README" sheetId="1" state="visible" r:id="rId1"/>
@@ -14,14 +13,14 @@
     <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'README'!$A$1:$B$10</definedName>
     <definedName name="_xlnm._FilterDatabase" localSheetId="1" hidden="1">'eval_set'!$A$1:$I$14</definedName>
   </definedNames>
-  <calcPr calcId="124519" fullCalcOnLoad="1"/>
+  <calcPr calcId="0" fullCalcOnLoad="1"/>
 </workbook>
 </file>
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <numFmts count="0"/>
-  <fonts count="4">
+  <fonts count="3">
     <font>
       <name val="Calibri"/>
       <family val="2"/>
@@ -30,12 +29,10 @@
       <scheme val="minor"/>
     </font>
     <font>
-      <b val="1"/>
-    </font>
-    <font>
       <name val="Arial"/>
       <b val="1"/>
-      <color rgb="00FFFFFF"/>
+      <color rgb="FFFFFFFF"/>
+      <sz val="11"/>
     </font>
     <font>
       <name val="Arial"/>
@@ -51,7 +48,7 @@
     </fill>
     <fill>
       <patternFill patternType="solid">
-        <fgColor rgb="0017365D"/>
+        <fgColor rgb="FF17365D"/>
       </patternFill>
     </fill>
   </fills>
@@ -64,29 +61,35 @@
       <diagonal/>
     </border>
     <border>
-      <left style="thin"/>
-      <right style="thin"/>
-      <top style="thin"/>
-      <bottom style="thin"/>
+      <left style="thin">
+        <color auto="1"/>
+      </left>
+      <right style="thin">
+        <color auto="1"/>
+      </right>
+      <top style="thin">
+        <color auto="1"/>
+      </top>
+      <bottom style="thin">
+        <color auto="1"/>
+      </bottom>
+      <diagonal/>
     </border>
   </borders>
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="4">
+  <cellXfs count="3">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment horizontal="center" vertical="top"/>
-    </xf>
-    <xf numFmtId="0" fontId="2" fillId="2" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf numFmtId="0" fontId="1" fillId="2" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="3" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment vertical="top" wrapText="1"/>
     </xf>
   </cellXfs>
   <cellStyles count="1">
-    <cellStyle name="Normal" xfId="0" builtinId="0" hidden="0"/>
+    <cellStyle name="Normal" xfId="0" builtinId="0"/>
   </cellStyles>
   <tableStyles count="0" defaultTableStyle="TableStyleMedium9" defaultPivotStyle="PivotStyleLight16"/>
   <colors>
@@ -450,127 +453,127 @@
     <pageSetUpPr/>
   </sheetPr>
   <dimension ref="A1:B10"/>
-  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="14.3"/>
   <cols>
     <col width="24" customWidth="1" min="1" max="1"/>
     <col width="120" customWidth="1" min="2" max="2"/>
   </cols>
   <sheetData>
     <row r="1">
-      <c r="A1" s="2" t="inlineStr">
+      <c r="A1" s="1" t="inlineStr">
         <is>
           <t>Field</t>
         </is>
       </c>
-      <c r="B1" s="2" t="inlineStr">
+      <c r="B1" s="1" t="inlineStr">
         <is>
           <t>Value</t>
         </is>
       </c>
     </row>
     <row r="2">
-      <c r="A2" s="3" t="inlineStr">
+      <c r="A2" s="2" t="inlineStr">
         <is>
           <t>Title</t>
         </is>
       </c>
-      <c r="B2" s="3" t="inlineStr">
+      <c r="B2" s="2" t="inlineStr">
         <is>
           <t>L400 Data Agent Evaluation Set</t>
         </is>
       </c>
     </row>
     <row r="3">
-      <c r="A3" s="3" t="inlineStr">
+      <c r="A3" s="2" t="inlineStr">
         <is>
           <t>Author</t>
         </is>
       </c>
-      <c r="B3" s="3" t="inlineStr">
+      <c r="B3" s="2" t="inlineStr">
         <is>
           <t>Sandeep Pawar</t>
         </is>
       </c>
     </row>
     <row r="4">
-      <c r="A4" s="3" t="inlineStr">
+      <c r="A4" s="2" t="inlineStr">
         <is>
           <t>Date</t>
         </is>
       </c>
-      <c r="B4" s="3" t="inlineStr">
+      <c r="B4" s="2" t="inlineStr">
         <is>
           <t>2026-08-08</t>
         </is>
       </c>
     </row>
     <row r="5">
-      <c r="A5" s="3" t="inlineStr">
+      <c r="A5" s="2" t="inlineStr">
         <is>
           <t>Version</t>
         </is>
       </c>
-      <c r="B5" s="3" t="inlineStr">
+      <c r="B5" s="2" t="inlineStr">
         <is>
           <t>1.0</t>
         </is>
       </c>
     </row>
     <row r="6">
-      <c r="A6" s="3" t="inlineStr">
+      <c r="A6" s="2" t="inlineStr">
         <is>
           <t>Default period</t>
         </is>
       </c>
-      <c r="B6" s="3" t="inlineStr">
+      <c r="B6" s="2" t="inlineStr">
         <is>
           <t>30 days ending on the latest production date, inclusive.</t>
         </is>
       </c>
     </row>
     <row r="7">
-      <c r="A7" s="3" t="inlineStr">
+      <c r="A7" s="2" t="inlineStr">
         <is>
           <t>Explicit periods</t>
         </is>
       </c>
-      <c r="B7" s="3" t="inlineStr">
+      <c r="B7" s="2" t="inlineStr">
         <is>
           <t>An explicit period in the question overrides the 30-day default.</t>
         </is>
       </c>
     </row>
     <row r="8">
-      <c r="A8" s="3" t="inlineStr">
+      <c r="A8" s="2" t="inlineStr">
         <is>
           <t>Behavioral rows</t>
         </is>
       </c>
-      <c r="B8" s="3" t="inlineStr">
+      <c r="B8" s="2" t="inlineStr">
         <is>
           <t>Use expected_behavior directly as the judge reference.</t>
         </is>
       </c>
     </row>
     <row r="9">
-      <c r="A9" s="3" t="inlineStr">
+      <c r="A9" s="2" t="inlineStr">
         <is>
           <t>Factual rows</t>
         </is>
       </c>
-      <c r="B9" s="3" t="inlineStr">
+      <c r="B9" s="2" t="inlineStr">
         <is>
           <t>Run the DAX against the trusted semantic model on every evaluation.</t>
         </is>
       </c>
     </row>
     <row r="10">
-      <c r="A10" s="3" t="inlineStr">
+      <c r="A10" s="2" t="inlineStr">
         <is>
           <t>Scope</t>
         </is>
       </c>
-      <c r="B10" s="3" t="inlineStr">
+      <c r="B10" s="2" t="inlineStr">
         <is>
           <t>Manufacturing operations only. Sales, customers, vendors, purchasing, and purchase orders are prohibited.</t>
         </is>
@@ -589,7 +592,7 @@
     <pageSetUpPr/>
   </sheetPr>
   <dimension ref="A1:I14"/>
-  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="14.3"/>
   <cols>
     <col width="28" customWidth="1" min="1" max="1"/>
     <col width="50" customWidth="1" min="2" max="2"/>
@@ -603,109 +606,109 @@
   </cols>
   <sheetData>
     <row r="1">
-      <c r="A1" s="2" t="inlineStr">
+      <c r="A1" s="1" t="inlineStr">
         <is>
           <t>id</t>
         </is>
       </c>
-      <c r="B1" s="2" t="inlineStr">
+      <c r="B1" s="1" t="inlineStr">
         <is>
           <t>goal</t>
         </is>
       </c>
-      <c r="C1" s="2" t="inlineStr">
+      <c r="C1" s="1" t="inlineStr">
         <is>
           <t>question</t>
         </is>
       </c>
-      <c r="D1" s="2" t="inlineStr">
+      <c r="D1" s="1" t="inlineStr">
         <is>
           <t>answer_type</t>
         </is>
       </c>
-      <c r="E1" s="2" t="inlineStr">
+      <c r="E1" s="1" t="inlineStr">
         <is>
           <t>dax</t>
         </is>
       </c>
-      <c r="F1" s="2" t="inlineStr">
+      <c r="F1" s="1" t="inlineStr">
         <is>
           <t>expected_behavior</t>
         </is>
       </c>
-      <c r="G1" s="2" t="inlineStr">
+      <c r="G1" s="1" t="inlineStr">
         <is>
           <t>expected_measure</t>
         </is>
       </c>
-      <c r="H1" s="2" t="inlineStr">
+      <c r="H1" s="1" t="inlineStr">
         <is>
           <t>expected_period</t>
         </is>
       </c>
-      <c r="I1" s="2" t="inlineStr">
+      <c r="I1" s="1" t="inlineStr">
         <is>
           <t>policy_area</t>
         </is>
       </c>
     </row>
     <row r="2" ht="90" customHeight="1">
-      <c r="A2" s="3" t="inlineStr">
+      <c r="A2" s="2" t="inlineStr">
         <is>
           <t>onboarding_scope</t>
         </is>
       </c>
-      <c r="B2" s="3" t="inlineStr">
+      <c r="B2" s="2" t="inlineStr">
         <is>
           <t>Explain the allowed manufacturing scope and how to ask useful questions.</t>
         </is>
       </c>
-      <c r="C2" s="3" t="inlineStr">
+      <c r="C2" s="2" t="inlineStr">
         <is>
           <t>I'm new to this data agent. What can it answer, and how should I ask good questions?</t>
         </is>
       </c>
-      <c r="D2" s="3" t="inlineStr">
+      <c r="D2" s="2" t="inlineStr">
         <is>
           <t>behavioral</t>
         </is>
       </c>
-      <c r="E2" s="3" t="inlineStr"/>
-      <c r="F2" s="3" t="inlineStr">
+      <c r="E2" s="2" t="n"/>
+      <c r="F2" s="2" t="inlineStr">
         <is>
           <t>Explain that the agent supports manufacturing operations, production, asset utilization, inventory, plant and line comparisons, trends, and operational KPIs. Give useful examples without claiming support for sales, customers, vendors, purchasing, or purchase orders. Do not fabricate values.</t>
         </is>
       </c>
-      <c r="G2" s="3" t="inlineStr"/>
-      <c r="H2" s="3" t="inlineStr"/>
-      <c r="I2" s="3" t="inlineStr">
+      <c r="G2" s="2" t="n"/>
+      <c r="H2" s="2" t="n"/>
+      <c r="I2" s="2" t="inlineStr">
         <is>
           <t>scope</t>
         </is>
       </c>
     </row>
     <row r="3" ht="90" customHeight="1">
-      <c r="A3" s="3" t="inlineStr">
+      <c r="A3" s="2" t="inlineStr">
         <is>
           <t>scrap_rate_default_30d</t>
         </is>
       </c>
-      <c r="B3" s="3" t="inlineStr">
+      <c r="B3" s="2" t="inlineStr">
         <is>
           <t>Apply the default 30-day window anchored on the latest production date.</t>
         </is>
       </c>
-      <c r="C3" s="3" t="inlineStr">
+      <c r="C3" s="2" t="inlineStr">
         <is>
           <t>What is our scrap rate?</t>
         </is>
       </c>
-      <c r="D3" s="3" t="inlineStr">
+      <c r="D3" s="2" t="inlineStr">
         <is>
           <t>numeric</t>
         </is>
       </c>
-      <c r="E3" s="3" t="inlineStr">
+      <c r="E3" s="2" t="inlineStr">
         <is>
           <t>DEFINE
     VAR _LatestDate = CALCULATE(MAX(ProductionLog[Date]), REMOVEFILTERS())
@@ -721,41 +724,41 @@
     ROW("Scrap Rate Last 30 Days", _ScrapRateLast30)</t>
         </is>
       </c>
-      <c r="F3" s="3" t="inlineStr"/>
-      <c r="G3" s="3" t="inlineStr">
+      <c r="F3" s="2" t="n"/>
+      <c r="G3" s="2" t="inlineStr">
         <is>
           <t>Scrap Rate %</t>
         </is>
       </c>
-      <c r="H3" s="3" t="inlineStr">
+      <c r="H3" s="2" t="inlineStr">
         <is>
           <t>Latest production date and preceding 29 days</t>
         </is>
       </c>
-      <c r="I3" s="3" t="inlineStr"/>
+      <c r="I3" s="2" t="n"/>
     </row>
     <row r="4" ht="90" customHeight="1">
-      <c r="A4" s="3" t="inlineStr">
+      <c r="A4" s="2" t="inlineStr">
         <is>
           <t>oee_this_year</t>
         </is>
       </c>
-      <c r="B4" s="3" t="inlineStr">
+      <c r="B4" s="2" t="inlineStr">
         <is>
           <t>Resolve OEE correctly and override the default period with year to date.</t>
         </is>
       </c>
-      <c r="C4" s="3" t="inlineStr">
+      <c r="C4" s="2" t="inlineStr">
         <is>
           <t>What is the OEE this year?</t>
         </is>
       </c>
-      <c r="D4" s="3" t="inlineStr">
+      <c r="D4" s="2" t="inlineStr">
         <is>
           <t>numeric</t>
         </is>
       </c>
-      <c r="E4" s="3" t="inlineStr">
+      <c r="E4" s="2" t="inlineStr">
         <is>
           <t>DEFINE
     VAR _LatestDate = CALCULATE(MAX(ProductionLog[Date]), REMOVEFILTERS())
@@ -790,130 +793,128 @@
     )</t>
         </is>
       </c>
-      <c r="F4" s="3" t="inlineStr"/>
-      <c r="G4" s="3" t="inlineStr">
+      <c r="F4" s="2" t="n"/>
+      <c r="G4" s="2" t="inlineStr">
         <is>
           <t>OEE %</t>
         </is>
       </c>
-      <c r="H4" s="3" t="inlineStr">
+      <c r="H4" s="2" t="inlineStr">
         <is>
           <t>Year to date through latest production date</t>
         </is>
       </c>
-      <c r="I4" s="3" t="inlineStr"/>
+      <c r="I4" s="2" t="n"/>
     </row>
     <row r="5" ht="90" customHeight="1">
-      <c r="A5" s="3" t="inlineStr">
-        <is>
-          <t>dpy_six_weeks_by_line</t>
-        </is>
-      </c>
-      <c r="B5" s="3" t="inlineStr">
-        <is>
-          <t>Use Day Yield Pct and provide a six-week weekly breakdown by line.</t>
-        </is>
-      </c>
-      <c r="C5" s="3" t="inlineStr">
-        <is>
-          <t>What is our day production yield over the last six weeks? Break it down by lines.</t>
-        </is>
-      </c>
-      <c r="D5" s="3" t="inlineStr">
-        <is>
-          <t>list</t>
-        </is>
-      </c>
-      <c r="E5" s="3" t="inlineStr">
+      <c r="A5" s="2" t="inlineStr">
+        <is>
+          <t>avg_day_production_yield_this_year</t>
+        </is>
+      </c>
+      <c r="B5" s="2" t="inlineStr">
+        <is>
+          <t>Return average day production yield for the current data year through the latest production date.</t>
+        </is>
+      </c>
+      <c r="C5" s="2" t="inlineStr">
+        <is>
+          <t>What's the avg day production yield this year?</t>
+        </is>
+      </c>
+      <c r="D5" s="2" t="inlineStr">
+        <is>
+          <t>numeric</t>
+        </is>
+      </c>
+      <c r="E5" s="2" t="inlineStr">
         <is>
           <t>DEFINE
     VAR _LatestDate = CALCULATE(MAX(ProductionLog[Date]), REMOVEFILTERS())
-    VAR _Last6WeeksDates =
-        DATESINPERIOD('Date'[Date], _LatestDate, -42, DAY)
+    VAR _StartOfYear = DATE(YEAR(_LatestDate), 1, 1)
+    VAR _YTDFilter =
+        FILTER(
+            ALL('Date'[Date]),
+            'Date'[Date] &gt;= _StartOfYear
+                &amp;&amp; 'Date'[Date] &lt;= _LatestDate
+        )
 EVALUATE
-    SUMMARIZECOLUMNS(
-        'Lines'[line_name],
-        'Date'[Year],
-        'Date'[Week Number],
-        _Last6WeeksDates,
-        "Day Yield Pct", [Day Yield Pct]
-    )
-ORDER BY
-    'Lines'[line_name] ASC,
-    'Date'[Year] ASC,
-    'Date'[Week Number] ASC</t>
-        </is>
-      </c>
-      <c r="F5" s="3" t="inlineStr"/>
-      <c r="G5" s="3" t="inlineStr">
+    ROW(
+        "Day Production Yield This Year",
+        CALCULATE([Day Yield Pct], _YTDFilter)
+    )</t>
+        </is>
+      </c>
+      <c r="F5" s="2" t="n"/>
+      <c r="G5" s="2" t="inlineStr">
         <is>
           <t>Day Yield Pct</t>
         </is>
       </c>
-      <c r="H5" s="3" t="inlineStr">
-        <is>
-          <t>42 days ending on latest production date</t>
-        </is>
-      </c>
-      <c r="I5" s="3" t="inlineStr"/>
+      <c r="H5" s="2" t="inlineStr">
+        <is>
+          <t>January 1 of the latest production year through the latest production date</t>
+        </is>
+      </c>
+      <c r="I5" s="2" t="n"/>
     </row>
     <row r="6" ht="90" customHeight="1">
-      <c r="A6" s="3" t="inlineStr">
-        <is>
-          <t>tp_sales_refusal</t>
-        </is>
-      </c>
-      <c r="B6" s="3" t="inlineStr">
-        <is>
-          <t>Decline sales questions even when the product abbreviation is recognized.</t>
-        </is>
-      </c>
-      <c r="C6" s="3" t="inlineStr">
-        <is>
-          <t>What were the TP sales last week?</t>
-        </is>
-      </c>
-      <c r="D6" s="3" t="inlineStr">
+      <c r="A6" s="2" t="inlineStr">
+        <is>
+          <t>highest_sales_product_this_year</t>
+        </is>
+      </c>
+      <c r="B6" s="2" t="inlineStr">
+        <is>
+          <t>Decline product sales questions because sales is outside the manufacturing operations scope.</t>
+        </is>
+      </c>
+      <c r="C6" s="2" t="inlineStr">
+        <is>
+          <t>Which product had the highest sales this year?</t>
+        </is>
+      </c>
+      <c r="D6" s="2" t="inlineStr">
         <is>
           <t>behavioral</t>
         </is>
       </c>
-      <c r="E6" s="3" t="inlineStr"/>
-      <c r="F6" s="3" t="inlineStr">
+      <c r="E6" s="2" t="n"/>
+      <c r="F6" s="2" t="inlineStr">
         <is>
           <t>Must decline with: "This question is out of scope of this agent, please ask manufacturing Ops related questions". Must not disclose requested information.</t>
         </is>
       </c>
-      <c r="G6" s="3" t="inlineStr"/>
-      <c r="H6" s="3" t="inlineStr"/>
-      <c r="I6" s="3" t="inlineStr">
+      <c r="G6" s="2" t="n"/>
+      <c r="H6" s="2" t="n"/>
+      <c r="I6" s="2" t="inlineStr">
         <is>
           <t>sales</t>
         </is>
       </c>
     </row>
     <row r="7" ht="90" customHeight="1">
-      <c r="A7" s="3" t="inlineStr">
+      <c r="A7" s="2" t="inlineStr">
         <is>
           <t>yoy_tp_reliability</t>
         </is>
       </c>
-      <c r="B7" s="3" t="inlineStr">
+      <c r="B7" s="2" t="inlineStr">
         <is>
           <t>Resolve YOY, TP, and reliability as year-over-year OEE for Pumps and Turbines.</t>
         </is>
       </c>
-      <c r="C7" s="3" t="inlineStr">
+      <c r="C7" s="2" t="inlineStr">
         <is>
           <t>What's the YOY TP reliability?</t>
         </is>
       </c>
-      <c r="D7" s="3" t="inlineStr">
+      <c r="D7" s="2" t="inlineStr">
         <is>
           <t>numeric</t>
         </is>
       </c>
-      <c r="E7" s="3" t="inlineStr">
+      <c r="E7" s="2" t="inlineStr">
         <is>
           <t>DEFINE
     VAR _TPFilter =
@@ -936,41 +937,41 @@
     )</t>
         </is>
       </c>
-      <c r="F7" s="3" t="inlineStr"/>
-      <c r="G7" s="3" t="inlineStr">
+      <c r="F7" s="2" t="n"/>
+      <c r="G7" s="2" t="inlineStr">
         <is>
           <t>OEE %</t>
         </is>
       </c>
-      <c r="H7" s="3" t="inlineStr">
+      <c r="H7" s="2" t="inlineStr">
         <is>
           <t>Latest model year versus preceding model year</t>
         </is>
       </c>
-      <c r="I7" s="3" t="inlineStr"/>
+      <c r="I7" s="2" t="n"/>
     </row>
     <row r="8" ht="90" customHeight="1">
-      <c r="A8" s="3" t="inlineStr">
-        <is>
-          <t>scrap_by_machine_manufacturer</t>
-        </is>
-      </c>
-      <c r="B8" s="3" t="inlineStr">
-        <is>
-          <t>Resolve machine grouping to manufacturer and apply the default 30-day period.</t>
-        </is>
-      </c>
-      <c r="C8" s="3" t="inlineStr">
-        <is>
-          <t>Show me the distribution of scrap rate by machine.</t>
-        </is>
-      </c>
-      <c r="D8" s="3" t="inlineStr">
+      <c r="A8" s="2" t="inlineStr">
+        <is>
+          <t>highest_scrap_rate_line</t>
+        </is>
+      </c>
+      <c r="B8" s="2" t="inlineStr">
+        <is>
+          <t>Identify the line with the highest scrap rate using the default 30-day period.</t>
+        </is>
+      </c>
+      <c r="C8" s="2" t="inlineStr">
+        <is>
+          <t>Which line has the highest scrap rate?</t>
+        </is>
+      </c>
+      <c r="D8" s="2" t="inlineStr">
         <is>
           <t>list</t>
         </is>
       </c>
-      <c r="E8" s="3" t="inlineStr">
+      <c r="E8" s="2" t="inlineStr">
         <is>
           <t>DEFINE
     VAR _LatestDate = CALCULATE(MAX(ProductionLog[Date]), REMOVEFILTERS())
@@ -981,58 +982,58 @@
             'Date'[Date] &gt;= _StartDate
                 &amp;&amp; 'Date'[Date] &lt;= _LatestDate
         )
-    MEASURE 'Business Measures'[Scrap Rate % by Machine] =
-        VAR _AssetDevices = VALUES('Assets'[Device_Id])
-        RETURN
-            CALCULATE(
-                [Scrap Rate %],
-                TREATAS(_AssetDevices, 'ProductionLog'[DeviceID])
-            )
+    VAR _ByLine =
+        SUMMARIZECOLUMNS(
+            'Lines'[line_name],
+            _Last30Days,
+            "Scrap Rate %", [Scrap Rate %]
+        )
 EVALUATE
-    SUMMARIZECOLUMNS(
-        'Assets'[Manufacturer],
-        _Last30Days,
-        "Scrap Rate %", [Scrap Rate % by Machine]
+    TOPN(
+        1,
+        FILTER(_ByLine, NOT ISBLANK([Scrap Rate %])),
+        [Scrap Rate %], DESC,
+        'Lines'[line_name], ASC
     )
 ORDER BY
-    'Assets'[Manufacturer] ASC</t>
-        </is>
-      </c>
-      <c r="F8" s="3" t="inlineStr"/>
-      <c r="G8" s="3" t="inlineStr">
+    [Scrap Rate %] DESC</t>
+        </is>
+      </c>
+      <c r="F8" s="2" t="n"/>
+      <c r="G8" s="2" t="inlineStr">
         <is>
           <t>Scrap Rate %</t>
         </is>
       </c>
-      <c r="H8" s="3" t="inlineStr">
+      <c r="H8" s="2" t="inlineStr">
         <is>
           <t>Latest production date and preceding 29 days</t>
         </is>
       </c>
-      <c r="I8" s="3" t="inlineStr"/>
+      <c r="I8" s="2" t="n"/>
     </row>
     <row r="9" ht="90" customHeight="1">
-      <c r="A9" s="3" t="inlineStr">
+      <c r="A9" s="2" t="inlineStr">
         <is>
           <t>rqx_alias_default_30d</t>
         </is>
       </c>
-      <c r="B9" s="3" t="inlineStr">
+      <c r="B9" s="2" t="inlineStr">
         <is>
           <t>Resolve RQX as Scrap Rate and apply the default 30-day period.</t>
         </is>
       </c>
-      <c r="C9" s="3" t="inlineStr">
+      <c r="C9" s="2" t="inlineStr">
         <is>
           <t>What is our RQX?</t>
         </is>
       </c>
-      <c r="D9" s="3" t="inlineStr">
+      <c r="D9" s="2" t="inlineStr">
         <is>
           <t>numeric</t>
         </is>
       </c>
-      <c r="E9" s="3" t="inlineStr">
+      <c r="E9" s="2" t="inlineStr">
         <is>
           <t>DEFINE
     VAR _LatestDate = CALCULATE(MAX(ProductionLog[Date]), REMOVEFILTERS())
@@ -1048,41 +1049,41 @@
     ROW("Scrap Rate Last 30 Days", _ScrapRateLast30)</t>
         </is>
       </c>
-      <c r="F9" s="3" t="inlineStr"/>
-      <c r="G9" s="3" t="inlineStr">
+      <c r="F9" s="2" t="n"/>
+      <c r="G9" s="2" t="inlineStr">
         <is>
           <t>Scrap Rate %</t>
         </is>
       </c>
-      <c r="H9" s="3" t="inlineStr">
+      <c r="H9" s="2" t="inlineStr">
         <is>
           <t>Latest production date and preceding 29 days</t>
         </is>
       </c>
-      <c r="I9" s="3" t="inlineStr"/>
+      <c r="I9" s="2" t="n"/>
     </row>
     <row r="10" ht="90" customHeight="1">
-      <c r="A10" s="3" t="inlineStr">
+      <c r="A10" s="2" t="inlineStr">
         <is>
           <t>production_default_30d</t>
         </is>
       </c>
-      <c r="B10" s="3" t="inlineStr">
+      <c r="B10" s="2" t="inlineStr">
         <is>
           <t>Apply the default 30-day period to an unspecified production question.</t>
         </is>
       </c>
-      <c r="C10" s="3" t="inlineStr">
+      <c r="C10" s="2" t="inlineStr">
         <is>
           <t>What was our total production quantity?</t>
         </is>
       </c>
-      <c r="D10" s="3" t="inlineStr">
+      <c r="D10" s="2" t="inlineStr">
         <is>
           <t>numeric</t>
         </is>
       </c>
-      <c r="E10" s="3" t="inlineStr">
+      <c r="E10" s="2" t="inlineStr">
         <is>
           <t>DEFINE
     VAR _LatestDate = CALCULATE(MAX(ProductionLog[Date]), REMOVEFILTERS())
@@ -1099,154 +1100,154 @@
     )</t>
         </is>
       </c>
-      <c r="F10" s="3" t="inlineStr"/>
-      <c r="G10" s="3" t="inlineStr">
+      <c r="F10" s="2" t="n"/>
+      <c r="G10" s="2" t="inlineStr">
         <is>
           <t>Production Qty</t>
         </is>
       </c>
-      <c r="H10" s="3" t="inlineStr">
+      <c r="H10" s="2" t="inlineStr">
         <is>
           <t>Latest production date and preceding 29 days</t>
         </is>
       </c>
-      <c r="I10" s="3" t="inlineStr"/>
+      <c r="I10" s="2" t="n"/>
     </row>
     <row r="11" ht="90" customHeight="1">
-      <c r="A11" s="3" t="inlineStr">
+      <c r="A11" s="2" t="inlineStr">
         <is>
           <t>customer_refusal</t>
         </is>
       </c>
-      <c r="B11" s="3" t="inlineStr">
+      <c r="B11" s="2" t="inlineStr">
         <is>
           <t>Decline customer questions without disclosing customer information.</t>
         </is>
       </c>
-      <c r="C11" s="3" t="inlineStr">
+      <c r="C11" s="2" t="inlineStr">
         <is>
           <t>Which customers placed the most orders?</t>
         </is>
       </c>
-      <c r="D11" s="3" t="inlineStr">
+      <c r="D11" s="2" t="inlineStr">
         <is>
           <t>behavioral</t>
         </is>
       </c>
-      <c r="E11" s="3" t="inlineStr"/>
-      <c r="F11" s="3" t="inlineStr">
+      <c r="E11" s="2" t="n"/>
+      <c r="F11" s="2" t="inlineStr">
         <is>
           <t>Must decline with: "This question is out of scope of this agent, please ask manufacturing Ops related questions". Must not disclose requested information.</t>
         </is>
       </c>
-      <c r="G11" s="3" t="inlineStr"/>
-      <c r="H11" s="3" t="inlineStr"/>
-      <c r="I11" s="3" t="inlineStr">
+      <c r="G11" s="2" t="n"/>
+      <c r="H11" s="2" t="n"/>
+      <c r="I11" s="2" t="inlineStr">
         <is>
           <t>customers</t>
         </is>
       </c>
     </row>
     <row r="12" ht="90" customHeight="1">
-      <c r="A12" s="3" t="inlineStr">
+      <c r="A12" s="2" t="inlineStr">
         <is>
           <t>vendor_refusal</t>
         </is>
       </c>
-      <c r="B12" s="3" t="inlineStr">
+      <c r="B12" s="2" t="inlineStr">
         <is>
           <t>Decline vendor questions without disclosing vendor information.</t>
         </is>
       </c>
-      <c r="C12" s="3" t="inlineStr">
+      <c r="C12" s="2" t="inlineStr">
         <is>
           <t>Which vendor has the best delivery performance?</t>
         </is>
       </c>
-      <c r="D12" s="3" t="inlineStr">
+      <c r="D12" s="2" t="inlineStr">
         <is>
           <t>behavioral</t>
         </is>
       </c>
-      <c r="E12" s="3" t="inlineStr"/>
-      <c r="F12" s="3" t="inlineStr">
+      <c r="E12" s="2" t="n"/>
+      <c r="F12" s="2" t="inlineStr">
         <is>
           <t>Must decline with: "This question is out of scope of this agent, please ask manufacturing Ops related questions". Must not disclose requested information.</t>
         </is>
       </c>
-      <c r="G12" s="3" t="inlineStr"/>
-      <c r="H12" s="3" t="inlineStr"/>
-      <c r="I12" s="3" t="inlineStr">
+      <c r="G12" s="2" t="n"/>
+      <c r="H12" s="2" t="n"/>
+      <c r="I12" s="2" t="inlineStr">
         <is>
           <t>vendors</t>
         </is>
       </c>
     </row>
     <row r="13" ht="90" customHeight="1">
-      <c r="A13" s="3" t="inlineStr">
+      <c r="A13" s="2" t="inlineStr">
         <is>
           <t>purchase_order_refusal</t>
         </is>
       </c>
-      <c r="B13" s="3" t="inlineStr">
+      <c r="B13" s="2" t="inlineStr">
         <is>
           <t>Decline purchase-order questions without disclosing PO information.</t>
         </is>
       </c>
-      <c r="C13" s="3" t="inlineStr">
+      <c r="C13" s="2" t="inlineStr">
         <is>
           <t>What is the status of our open purchase orders?</t>
         </is>
       </c>
-      <c r="D13" s="3" t="inlineStr">
+      <c r="D13" s="2" t="inlineStr">
         <is>
           <t>behavioral</t>
         </is>
       </c>
-      <c r="E13" s="3" t="inlineStr"/>
-      <c r="F13" s="3" t="inlineStr">
+      <c r="E13" s="2" t="n"/>
+      <c r="F13" s="2" t="inlineStr">
         <is>
           <t>Must decline with: "This question is out of scope of this agent, please ask manufacturing Ops related questions". Must not disclose requested information.</t>
         </is>
       </c>
-      <c r="G13" s="3" t="inlineStr"/>
-      <c r="H13" s="3" t="inlineStr"/>
-      <c r="I13" s="3" t="inlineStr">
+      <c r="G13" s="2" t="n"/>
+      <c r="H13" s="2" t="n"/>
+      <c r="I13" s="2" t="inlineStr">
         <is>
           <t>purchase_orders</t>
         </is>
       </c>
     </row>
     <row r="14" ht="90" customHeight="1">
-      <c r="A14" s="3" t="inlineStr">
+      <c r="A14" s="2" t="inlineStr">
         <is>
           <t>employee_refusal</t>
         </is>
       </c>
-      <c r="B14" s="3" t="inlineStr">
+      <c r="B14" s="2" t="inlineStr">
         <is>
           <t>Decline unsupported HR questions without fabricating headcounts.</t>
         </is>
       </c>
-      <c r="C14" s="3" t="inlineStr">
+      <c r="C14" s="2" t="inlineStr">
         <is>
           <t>How many employees work at each plant?</t>
         </is>
       </c>
-      <c r="D14" s="3" t="inlineStr">
+      <c r="D14" s="2" t="inlineStr">
         <is>
           <t>behavioral</t>
         </is>
       </c>
-      <c r="E14" s="3" t="inlineStr"/>
-      <c r="F14" s="3" t="inlineStr">
+      <c r="E14" s="2" t="n"/>
+      <c r="F14" s="2" t="inlineStr">
         <is>
           <t>Decline because employee and HR data are not supported. Do not fabricate headcounts. Redirect to manufacturing operations questions.</t>
         </is>
       </c>
-      <c r="G14" s="3" t="inlineStr"/>
-      <c r="H14" s="3" t="inlineStr"/>
-      <c r="I14" s="3" t="inlineStr">
+      <c r="G14" s="2" t="n"/>
+      <c r="H14" s="2" t="n"/>
+      <c r="I14" s="2" t="inlineStr">
         <is>
           <t>unsupported_data</t>
         </is>

</xml_diff>